<commit_message>
Add tutorial audio, escape task, and lighting visibility
</commit_message>
<xml_diff>
--- a/outputs/comment_task_flow_template/コメント・タスク進行表_テンプレート.xlsx
+++ b/outputs/comment_task_flow_template/コメント・タスク進行表_テンプレート.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\gameseisaku\GCCC2026_GroupB\outputs\comment_task_flow_template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BA5E977-DAA2-413E-AA72-232166054F74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC13939E-2E9F-44C2-B910-969DCC83F79C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="177">
   <si>
     <t>コメント・タスク進行定義表</t>
   </si>
@@ -1034,6 +1034,27 @@
     </rPh>
     <rPh sb="7" eb="9">
       <t>テントウ</t>
+    </rPh>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>16</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>脱出せよ</t>
+    <rPh sb="0" eb="2">
+      <t>ダッシュツ</t>
+    </rPh>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>このタスクが始まるとゴールが解放される</t>
+    <rPh sb="6" eb="7">
+      <t>ハジ</t>
+    </rPh>
+    <rPh sb="14" eb="16">
+      <t>カイホウ</t>
     </rPh>
     <phoneticPr fontId="5"/>
   </si>
@@ -2414,23 +2435,37 @@
         <v>171</v>
       </c>
     </row>
-    <row r="24" spans="1:16">
-      <c r="A24" s="13"/>
-      <c r="B24" s="14"/>
-      <c r="C24" s="14"/>
+    <row r="24" spans="1:16" ht="28.5">
+      <c r="A24" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="B24" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="C24" s="14" t="s">
+        <v>175</v>
+      </c>
       <c r="D24" s="14"/>
       <c r="E24" s="15"/>
-      <c r="F24" s="14"/>
-      <c r="G24" s="15"/>
+      <c r="F24" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="G24" s="15" t="s">
+        <v>168</v>
+      </c>
       <c r="H24" s="14"/>
       <c r="I24" s="14"/>
       <c r="J24" s="14"/>
       <c r="K24" s="14"/>
       <c r="L24" s="14"/>
-      <c r="M24" s="16"/>
+      <c r="M24" s="16">
+        <v>0</v>
+      </c>
       <c r="N24" s="15"/>
       <c r="O24" s="15"/>
-      <c r="P24" s="17"/>
+      <c r="P24" s="17" t="s">
+        <v>176</v>
+      </c>
     </row>
     <row r="25" spans="1:16">
       <c r="A25" s="13"/>

</xml_diff>